<commit_message>
Rebuild CBRS on risk-adjusted OpenAI ramp after UBS initiation
UBS (8 Jun 2026) initiated Buy/$300, surfacing an OpenAI 750MW prepayment
deal and an AWS disaggregated-inference program that the original skills-only
model missed. Rebuild base case on a risk-adjusted OpenAI ramp (~12mo behind
UBS, ~55-60% utilization); AWS treated as bull-only optionality.

Blended target $51 -> $134 (-43.7%). Bull scenario $255 lands near UBS $300;
remaining gap is execution-risk weighting, not a data dispute.
</commit_message>
<xml_diff>
--- a/output/CBRS/CBRS.xlsx
+++ b/output/CBRS/CBRS.xlsx
@@ -574,7 +574,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>$51.00</t>
+          <t>$134</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>-78.7%</t>
+          <t>-43.7%</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>$50.64</t>
+          <t>$134</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>-78.7%</t>
+          <t>-43.7%</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>n/a (data gap)</t>
+          <t>$300 (UBS, sole initiation seen)</t>
         </is>
       </c>
     </row>
@@ -806,7 +806,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>$34.69</t>
+          <t>$119</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>$109</t>
+          <t>$193</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Real technology, wrong price: Cerebras owns the only wafer-scale chip in production and the fastest published inference benchmarks, and revenue compounded from $24.6M (2022) to $510M (2025). None of that justifies 102x trailing sales.</t>
+          <t>Real franchise, now with a real anchor: the UBS initiation surfaced an OpenAI 750MW prepayment deal (~$20B+ over its life, expandable to 2GW) plus an AWS disaggregated-inference program. Our prior skills-only model missed both; rebuilt for them, fair value rises from $51 to about $134.</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>A long-horizon FCFF DCF on a constructive ramp (revenue to ~$5.5B by 2035, FCF margin to 25%) values the equity near $35 base case; even a generous 28x FY26E sales cross-check lands near $110. Spot is $238.</t>
+          <t>The gap to spot is execution timing, not technology. Base case risk-adjusts the OpenAI ramp ~12 months behind UBS at ~55-60% utilization (the supply chain must scale roughly 10x) and excludes AWS; that path is worth ~$119. If OpenAI ramps on schedule and AWS converts, the bull case reaches ~$255, near UBS's $300.</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>The downside catalysts are concrete and dateable: an IPO lock-up unlock against a 8.67M-share float, ~85% single-customer (G42) revenue concentration, and US export-control exposure on Gulf compute.</t>
+          <t>At $238 the market already credits the UBS-style on-schedule outcome. Blended fair value $134 (-43.7%) says pay less or wait for proof of the ramp; the lock-up unlock and OpenAI concentration are the swing risks.</t>
         </is>
       </c>
     </row>
@@ -942,7 +942,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>DCF — Cerebras is loss-making today but has a clear revenue ramp, improving gross margin and a fixed R&amp;D base that scales into profit. A long-horizon FCFF DCF captures the path to cash generation better than a trailing multiple; an EV/Sales cross-check anchors the near-term sanity check given the 102x trailing-sales valuation.</t>
+          <t>DCF — After the UBS initiation surfaced the OpenAI 750MW prepayment deal and the AWS disaggregated-inference program (neither in our prior skills-only model), we rebuild the base on a risk-adjusted OpenAI ramp: ~12 months behind UBS and at ~55-60% of their modeled capacity, reflecting the ~10x supply-chain scale-up required. AWS is excluded from the base and treated as bull-case upside. A long-horizon FCFF DCF captures the path to OpenAI-driven profitability; an EV/Sales cross-check on forward sales anchors it against hardware peers.</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Ke = 4.4% Rf + 1.30 beta x 5.5% ERP = 11.6%. Beta set above the semi average for single-architecture concentration, ~85% single-customer revenue and post-IPO volatility (49% peak-to-trough in year one). Net cash means debt weight ~1%, so WACC sits near Ke at 11.5%, inside the 9-12% semi band.</t>
+          <t>Ke = 4.4% Rf + 1.30 beta x 5.5% ERP = 11.6%. Beta above the semi average for OpenAI single-customer concentration (now the anchor, replacing G42), the 10x supply-chain execution risk, and post-IPO volatility. Net cash keeps debt weight ~1%, so WACC ~11.5%, inside the 9-12% semi band.</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Inference compute should outgrow GDP for years; 3.5% terminal is defensible for a durable franchise but below the early ramp.</t>
+          <t>Inference compute outgrows GDP for years; 3.5% terminal for a durable franchise, below the explicit ramp.</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Multiple — EV/Sales is the standard cross-check for loss-making hypergrowth. Peer set: high-growth AI compute and inference names. A rich 28x FY26E sales is generous versus where most AI hardware trades, and still implies a price far below the current $237.83, underscoring how stretched the trailing 102x multiple is.</t>
+          <t>Multiple — UBS values CBRS at 10x EV/Sales on C2029E sales discounted back. We apply the same compute-peer ~10x multiple but to our risk-adjusted C2028E sales of $4.2B, undiscounted, as a ~18-month forward target proxy. This stays conservative versus UBS (lower year, lower sales) while using the same relative lens the market is using.</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Base 45% reflects a constructive but realistic ramp. Bear gets a heavy 20% because the lock-up unlock, G42 concentration and export risk are concrete near-term catalysts, not tail events. Bull 15% for the demand-reacceleration case. The EV/Sales cross-check carries 20% to anchor against intrinsic value with a relative lens; notably even a generous 28x sales multiple lands well below spot, which is the central finding.</t>
+          <t>Base 45% on the risk-adjusted OpenAI ramp. Bear gets a heavy 25% because the 10x supply-chain scale-up, OpenAI concentration, NVDA/Groq competitive response, and the IPO lock-up are all live. Bull 20% for the OpenAI-on-schedule-plus-AWS case. Cross-check 10% as a hardware-peer relative anchor. The blend deliberately stays below UBS's $300 by haircutting the deal for execution rather than disputing the technology.</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>No sell-side consensus, mean/median price target, or analyst count returned by yfinance. | FY25 segment split between hardware (systems/supercomputers) and inference cloud not in the available data; needs the 10-K segment note. | Exact FY25 G42 revenue concentration (was ~83-87% in the 2023 S-1); needs the latest 10-K footnote. | Beta not available from yfinance; WACC beta of 1.30 is an analyst estimate reflecting concentration and post-IPO volatility. | IPO lock-up expiry date not retrievable via available skills; flagged as the key catalyst. | Reported FY25 free cash flow figure is distorted by customer prepayments; treat operating-CF-near-breakeven with caution.</t>
+          <t>OpenAI and AWS deal terms are sourced from the UBS initiation (8 Jun 2026), not a primary CBRS filing; our base risk-adjusts UBS's schedule. | Exact OpenAI tranche timing and pricing not independently verified; modeled at ~55-60% of UBS utilization, ~12 months behind. | AWS program is unsized (pilot stage); excluded from base, modeled only in the bull scenario. | FY25 segment split (hardware vs inference cloud) still not in primary data. | IPO lock-up expiry date not retrievable via available skills; flagged as a key catalyst. | Beta not available from yfinance; WACC beta 1.30 is an analyst estimate for concentration and post-IPO volatility.</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Thin / none returned</t>
+          <t>UBS: Buy, $300 PT (8 Jun 2026)</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>n/a (data gap)</t>
+          <t>$300 (UBS, sole initiation seen)</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>$51 (-78.7%)</t>
+          <t>$134 (-43.7%)</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Ke = 4.4% Rf + 1.30 beta x 5.5% ERP = 11.6%. Beta set above the semi average for single-architecture concentration, ~85% single-customer revenue and post-IPO volatility (49% peak-to-trough in year one). Net cash means debt weight ~1%, so WACC sits near Ke at 11.5%, inside the 9-12% semi band.</t>
+          <t>Ke = 4.4% Rf + 1.30 beta x 5.5% ERP = 11.6%. Beta above the semi average for OpenAI single-customer concentration (now the anchor, replacing G42), the 10x supply-chain execution risk, and post-IPO volatility. Net cash keeps debt weight ~1%, so WACC ~11.5%, inside the 9-12% semi band.</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Inference compute should outgrow GDP for years; 3.5% terminal is defensible for a durable franchise but below the early ramp.</t>
+          <t>Inference compute outgrows GDP for years; 3.5% terminal for a durable franchise, below the explicit ramp.</t>
         </is>
       </c>
     </row>
@@ -1829,14 +1829,14 @@
         <v>2026</v>
       </c>
       <c r="B16" t="n">
-        <v>-0.1599</v>
+        <v>-0.4116</v>
       </c>
       <c r="C16" t="n">
-        <v>0.8415</v>
+        <v>0.84</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>FY26E +65%: inference cloud scaling plus Condor Galaxy installs; growth decelerates off the 2025 76% print. Still operating-loss as R&amp;D base dominates.</t>
+          <t>C2026E ~$0.84B: in line with UBS ($0.83B) and our prior model. Near-term visibility is good; OpenAI contributes little this year as the first 250MW tranche only begins to deploy.</t>
         </is>
       </c>
     </row>
@@ -1845,14 +1845,14 @@
         <v>2027</v>
       </c>
       <c r="B17" t="n">
-        <v>-0.1199</v>
+        <v>-0.1949</v>
       </c>
       <c r="C17" t="n">
-        <v>1.2622</v>
+        <v>1.9</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>FY27E +50%: enterprise and sovereign pipeline broadens; gross margin lifts on cloud mix; loss narrows toward breakeven.</t>
+          <t>C2027E +126% to $1.9B vs UBS $2.70B. OpenAI tranche-1 deployment begins but we haircut ~30% for the 10x supply-chain scale-up. AWS excluded from base.</t>
         </is>
       </c>
     </row>
@@ -1861,14 +1861,14 @@
         <v>2028</v>
       </c>
       <c r="B18" t="n">
-        <v>-0.0223</v>
+        <v>0.268</v>
       </c>
       <c r="C18" t="n">
-        <v>1.7671</v>
+        <v>4.2</v>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>FY28E +40%: first year of positive operating margin as revenue laps the fixed R&amp;D base.</t>
+          <t>C2028E +121% to $4.2B vs UBS $7.12B (~59% of UBS). Peak OpenAI tranche-1 ramp, risk-adjusted for slippage. Still no AWS credit.</t>
         </is>
       </c>
     </row>
@@ -1877,14 +1877,14 @@
         <v>2029</v>
       </c>
       <c r="B19" t="n">
-        <v>0.1162</v>
+        <v>0.9828</v>
       </c>
       <c r="C19" t="n">
-        <v>2.3326</v>
+        <v>6.5</v>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>FY29E +32%: operating leverage builds; capex intensity easing as the manufacturing base matures.</t>
+          <t>C2029E +55% to $6.5B vs UBS $11.16B (~58%). Tranches layer in but a year behind UBS schedule; concentration on OpenAI is now the key risk.</t>
         </is>
       </c>
     </row>
@@ -1893,14 +1893,14 @@
         <v>2030</v>
       </c>
       <c r="B20" t="n">
-        <v>0.3041</v>
+        <v>1.6566</v>
       </c>
       <c r="C20" t="n">
-        <v>2.9158</v>
+        <v>8.5</v>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>FY30E +25%: mid-teens FCF margin as cloud mix and pricing stabilize.</t>
+          <t>C2030E +31% to $8.5B vs UBS $15.55B (~55%). Mature OpenAI footprint at risk-adjusted utilization.</t>
         </is>
       </c>
     </row>
@@ -1909,14 +1909,14 @@
         <v>2031</v>
       </c>
       <c r="B21" t="n">
-        <v>0.4829</v>
+        <v>2.2216</v>
       </c>
       <c r="C21" t="n">
-        <v>3.499</v>
+        <v>10.2</v>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>FY31E +20%: franchise scaling; FCF margin high-teens.</t>
+          <t>C2031E +20% to $10.2B: deceleration as the 750MW base fills; optional 2GW expansion and AWS sit in the bull case, not here.</t>
         </is>
       </c>
     </row>
@@ -1925,14 +1925,14 @@
         <v>2032</v>
       </c>
       <c r="B22" t="n">
-        <v>0.7171999999999999</v>
+        <v>2.7577</v>
       </c>
       <c r="C22" t="n">
-        <v>4.0588</v>
+        <v>11.7</v>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>FY32E +16%: deceleration continues off a larger base.</t>
+          <t>C2032E +15% to $11.7B: franchise scaling past the initial OpenAI commitment.</t>
         </is>
       </c>
     </row>
@@ -1941,14 +1941,14 @@
         <v>2033</v>
       </c>
       <c r="B23" t="n">
-        <v>0.8829</v>
+        <v>3.2842</v>
       </c>
       <c r="C23" t="n">
-        <v>4.5864</v>
+        <v>13.1</v>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>FY33E +13%: maturing growth, low-20s FCF margin.</t>
+          <t>C2033E +12% to $13.1B: maturing growth.</t>
         </is>
       </c>
     </row>
@@ -1957,14 +1957,14 @@
         <v>2034</v>
       </c>
       <c r="B24" t="n">
-        <v>1.0966</v>
+        <v>3.698</v>
       </c>
       <c r="C24" t="n">
-        <v>5.0909</v>
+        <v>14.3</v>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>FY34E +11%: approaching steady state.</t>
+          <t>C2034E +9% to $14.3B: approaching steady state.</t>
         </is>
       </c>
     </row>
@@ -1973,14 +1973,14 @@
         <v>2035</v>
       </c>
       <c r="B25" t="n">
-        <v>1.2391</v>
+        <v>4.1096</v>
       </c>
       <c r="C25" t="n">
-        <v>5.5491</v>
+        <v>15.3</v>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>FY35E +9%: terminal-approach year, ~25% FCF margin franchise.</t>
+          <t>C2035E +7% to $15.3B: terminal-approach year, hardware-like ~34% EBIT margin.</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2207,7 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>11.5% is mid-to-upper semi band; justified by concentration and float risk.</t>
+          <t>11.5% mid-upper semi band; concentration shifts from G42 to OpenAI but remains high.</t>
         </is>
       </c>
     </row>
@@ -2283,34 +2283,34 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.842</v>
+        <v>0.84</v>
       </c>
       <c r="C21" t="n">
-        <v>1.262</v>
+        <v>1.9</v>
       </c>
       <c r="D21" t="n">
-        <v>1.767</v>
+        <v>4.2</v>
       </c>
       <c r="E21" t="n">
-        <v>2.333</v>
+        <v>6.5</v>
       </c>
       <c r="F21" t="n">
-        <v>2.916</v>
+        <v>8.5</v>
       </c>
       <c r="G21" t="n">
-        <v>3.499</v>
+        <v>10.2</v>
       </c>
       <c r="H21" t="n">
-        <v>4.059</v>
+        <v>11.7</v>
       </c>
       <c r="I21" t="n">
-        <v>4.586</v>
+        <v>13.1</v>
       </c>
       <c r="J21" t="n">
-        <v>5.091</v>
+        <v>14.3</v>
       </c>
       <c r="K21" t="n">
-        <v>5.549</v>
+        <v>15.3</v>
       </c>
     </row>
     <row r="22">
@@ -2319,35 +2319,37 @@
           <t>YoY growth</t>
         </is>
       </c>
-      <c r="B22" s="11" t="n">
-        <v>0.65</v>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>0.5</v>
+        <v>1.262</v>
       </c>
       <c r="D22" s="11" t="n">
-        <v>0.4</v>
+        <v>1.211</v>
       </c>
       <c r="E22" s="11" t="n">
-        <v>0.32</v>
+        <v>0.5479999999999999</v>
       </c>
       <c r="F22" s="11" t="n">
-        <v>0.25</v>
+        <v>0.308</v>
       </c>
       <c r="G22" s="11" t="n">
         <v>0.2</v>
       </c>
       <c r="H22" s="11" t="n">
-        <v>0.16</v>
+        <v>0.147</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>0.11</v>
+        <v>0.092</v>
       </c>
       <c r="K22" s="11" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="23">
@@ -2357,34 +2359,34 @@
         </is>
       </c>
       <c r="B23" s="11" t="n">
-        <v>-0.1</v>
+        <v>-0.3</v>
       </c>
       <c r="C23" s="11" t="n">
-        <v>-0.02</v>
+        <v>0.06</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>0.06</v>
+        <v>0.22</v>
       </c>
       <c r="E23" s="11" t="n">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>0.17</v>
+        <v>0.31</v>
       </c>
       <c r="G23" s="11" t="n">
-        <v>0.2</v>
+        <v>0.32</v>
       </c>
       <c r="H23" s="11" t="n">
-        <v>0.23</v>
+        <v>0.33</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>0.25</v>
+        <v>0.33</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>0.26</v>
+        <v>0.34</v>
       </c>
       <c r="K23" s="11" t="n">
-        <v>0.27</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="24">
@@ -2394,34 +2396,34 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.08400000000000001</v>
+        <v>-0.252</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.025</v>
+        <v>0.114</v>
       </c>
       <c r="D24" t="n">
-        <v>0.106</v>
+        <v>0.924</v>
       </c>
       <c r="E24" t="n">
-        <v>0.28</v>
+        <v>1.82</v>
       </c>
       <c r="F24" t="n">
-        <v>0.496</v>
+        <v>2.635</v>
       </c>
       <c r="G24" t="n">
-        <v>0.7</v>
+        <v>3.264</v>
       </c>
       <c r="H24" t="n">
-        <v>0.9340000000000001</v>
+        <v>3.861</v>
       </c>
       <c r="I24" t="n">
-        <v>1.147</v>
+        <v>4.323</v>
       </c>
       <c r="J24" t="n">
-        <v>1.324</v>
+        <v>4.862</v>
       </c>
       <c r="K24" t="n">
-        <v>1.498</v>
+        <v>5.202</v>
       </c>
     </row>
     <row r="25">
@@ -2468,34 +2470,34 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>-0.066</v>
+        <v>-0.199</v>
       </c>
       <c r="C26" t="n">
-        <v>-0.02</v>
+        <v>0.09</v>
       </c>
       <c r="D26" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.73</v>
       </c>
       <c r="E26" t="n">
-        <v>0.221</v>
+        <v>1.438</v>
       </c>
       <c r="F26" t="n">
-        <v>0.392</v>
+        <v>2.082</v>
       </c>
       <c r="G26" t="n">
-        <v>0.553</v>
+        <v>2.579</v>
       </c>
       <c r="H26" t="n">
-        <v>0.737</v>
+        <v>3.05</v>
       </c>
       <c r="I26" t="n">
-        <v>0.906</v>
+        <v>3.415</v>
       </c>
       <c r="J26" t="n">
-        <v>1.046</v>
+        <v>3.841</v>
       </c>
       <c r="K26" t="n">
-        <v>1.184</v>
+        <v>4.11</v>
       </c>
     </row>
     <row r="27">
@@ -2505,34 +2507,34 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.059</v>
+        <v>0.067</v>
       </c>
       <c r="C27" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.152</v>
       </c>
       <c r="D27" t="n">
-        <v>0.124</v>
+        <v>0.336</v>
       </c>
       <c r="E27" t="n">
-        <v>0.163</v>
+        <v>0.52</v>
       </c>
       <c r="F27" t="n">
-        <v>0.204</v>
+        <v>0.68</v>
       </c>
       <c r="G27" t="n">
-        <v>0.245</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="H27" t="n">
-        <v>0.284</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="I27" t="n">
-        <v>0.321</v>
+        <v>1.048</v>
       </c>
       <c r="J27" t="n">
-        <v>0.356</v>
+        <v>1.144</v>
       </c>
       <c r="K27" t="n">
-        <v>0.388</v>
+        <v>1.224</v>
       </c>
     </row>
     <row r="28">
@@ -2542,34 +2544,34 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.101</v>
+        <v>0.21</v>
       </c>
       <c r="C28" t="n">
-        <v>0.139</v>
+        <v>0.38</v>
       </c>
       <c r="D28" t="n">
-        <v>0.177</v>
+        <v>0.672</v>
       </c>
       <c r="E28" t="n">
-        <v>0.21</v>
+        <v>0.845</v>
       </c>
       <c r="F28" t="n">
-        <v>0.233</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="G28" t="n">
-        <v>0.245</v>
+        <v>1.02</v>
       </c>
       <c r="H28" t="n">
-        <v>0.244</v>
+        <v>1.053</v>
       </c>
       <c r="I28" t="n">
-        <v>0.275</v>
+        <v>1.048</v>
       </c>
       <c r="J28" t="n">
-        <v>0.255</v>
+        <v>1.144</v>
       </c>
       <c r="K28" t="n">
-        <v>0.277</v>
+        <v>1.071</v>
       </c>
     </row>
     <row r="29">
@@ -2579,34 +2581,34 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.034</v>
+        <v>0.017</v>
       </c>
       <c r="C29" t="n">
-        <v>0.044</v>
+        <v>0.057</v>
       </c>
       <c r="D29" t="n">
-        <v>0.053</v>
+        <v>0.126</v>
       </c>
       <c r="E29" t="n">
-        <v>0.058</v>
+        <v>0.13</v>
       </c>
       <c r="F29" t="n">
-        <v>0.058</v>
+        <v>0.17</v>
       </c>
       <c r="G29" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.153</v>
       </c>
       <c r="H29" t="n">
-        <v>0.061</v>
+        <v>0.175</v>
       </c>
       <c r="I29" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.131</v>
       </c>
       <c r="J29" t="n">
-        <v>0.051</v>
+        <v>0.143</v>
       </c>
       <c r="K29" t="n">
-        <v>0.055</v>
+        <v>0.153</v>
       </c>
     </row>
     <row r="30">
@@ -2616,34 +2618,34 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>-0.16</v>
+        <v>-0.412</v>
       </c>
       <c r="C30" t="n">
-        <v>-0.12</v>
+        <v>-0.195</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.022</v>
+        <v>0.268</v>
       </c>
       <c r="E30" t="n">
-        <v>0.116</v>
+        <v>0.983</v>
       </c>
       <c r="F30" t="n">
-        <v>0.304</v>
+        <v>1.657</v>
       </c>
       <c r="G30" t="n">
-        <v>0.483</v>
+        <v>2.222</v>
       </c>
       <c r="H30" t="n">
-        <v>0.717</v>
+        <v>2.758</v>
       </c>
       <c r="I30" t="n">
-        <v>0.883</v>
+        <v>3.284</v>
       </c>
       <c r="J30" t="n">
-        <v>1.097</v>
+        <v>3.698</v>
       </c>
       <c r="K30" t="n">
-        <v>1.239</v>
+        <v>4.11</v>
       </c>
     </row>
     <row r="31">
@@ -2690,34 +2692,34 @@
         </is>
       </c>
       <c r="B32" s="16" t="n">
-        <v>-0.143</v>
+        <v>-0.369</v>
       </c>
       <c r="C32" s="16" t="n">
-        <v>-0.096</v>
+        <v>-0.157</v>
       </c>
       <c r="D32" s="16" t="n">
-        <v>-0.016</v>
+        <v>0.193</v>
       </c>
       <c r="E32" s="16" t="n">
-        <v>0.075</v>
+        <v>0.636</v>
       </c>
       <c r="F32" s="16" t="n">
-        <v>0.176</v>
+        <v>0.961</v>
       </c>
       <c r="G32" s="16" t="n">
-        <v>0.251</v>
+        <v>1.156</v>
       </c>
       <c r="H32" s="16" t="n">
-        <v>0.335</v>
+        <v>1.287</v>
       </c>
       <c r="I32" s="16" t="n">
-        <v>0.37</v>
+        <v>1.375</v>
       </c>
       <c r="J32" s="16" t="n">
-        <v>0.412</v>
+        <v>1.388</v>
       </c>
       <c r="K32" s="16" t="n">
-        <v>0.417</v>
+        <v>1.384</v>
       </c>
     </row>
     <row r="33"/>
@@ -2745,7 +2747,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1.2391</v>
+        <v>4.1096</v>
       </c>
     </row>
     <row r="37">
@@ -2755,17 +2757,17 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>16.03085625</v>
+        <v>53.16795</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>TV — Exit multiple (18.0× EBITDA, bn)</t>
+          <t>TV — Exit multiple (16.0× EBITDA, bn)</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>33.960492</v>
+        <v>102.816</v>
       </c>
     </row>
     <row r="39">
@@ -2775,7 +2777,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>24.995674125</v>
+        <v>77.99197500000001</v>
       </c>
     </row>
     <row r="40">
@@ -2785,7 +2787,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>5.397691334717424</v>
+        <v>17.90198717549409</v>
       </c>
     </row>
     <row r="41">
@@ -2795,7 +2797,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>8.416202573704261</v>
+        <v>26.2603943962755</v>
       </c>
     </row>
     <row r="42"/>
@@ -2806,7 +2808,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1.78</v>
+        <v>7.855</v>
       </c>
     </row>
     <row r="44">
@@ -2816,7 +2818,7 @@
         </is>
       </c>
       <c r="B44" s="16" t="n">
-        <v>7.178</v>
+        <v>25.757</v>
       </c>
     </row>
     <row r="45">
@@ -2836,7 +2838,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>7.617</v>
+        <v>26.196</v>
       </c>
     </row>
     <row r="47">
@@ -2857,7 +2859,7 @@
         </is>
       </c>
       <c r="B49" s="19" t="n">
-        <v>34.69</v>
+        <v>119.29</v>
       </c>
     </row>
   </sheetData>
@@ -3060,13 +3062,13 @@
         <v>2026</v>
       </c>
       <c r="B16" t="n">
-        <v>-0.16</v>
+        <v>-0.412</v>
       </c>
       <c r="C16" t="n">
         <v>0.8969</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.143</v>
+        <v>-0.369</v>
       </c>
     </row>
     <row r="17">
@@ -3074,13 +3076,13 @@
         <v>2027</v>
       </c>
       <c r="B17" t="n">
-        <v>-0.12</v>
+        <v>-0.195</v>
       </c>
       <c r="C17" t="n">
         <v>0.8044</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.096</v>
+        <v>-0.157</v>
       </c>
     </row>
     <row r="18">
@@ -3088,13 +3090,13 @@
         <v>2028</v>
       </c>
       <c r="B18" t="n">
-        <v>-0.022</v>
+        <v>0.268</v>
       </c>
       <c r="C18" t="n">
         <v>0.7214</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.016</v>
+        <v>0.193</v>
       </c>
     </row>
     <row r="19">
@@ -3102,13 +3104,13 @@
         <v>2029</v>
       </c>
       <c r="B19" t="n">
-        <v>0.116</v>
+        <v>0.983</v>
       </c>
       <c r="C19" t="n">
         <v>0.647</v>
       </c>
       <c r="D19" t="n">
-        <v>0.075</v>
+        <v>0.636</v>
       </c>
     </row>
     <row r="20">
@@ -3116,13 +3118,13 @@
         <v>2030</v>
       </c>
       <c r="B20" t="n">
-        <v>0.304</v>
+        <v>1.657</v>
       </c>
       <c r="C20" t="n">
         <v>0.5803</v>
       </c>
       <c r="D20" t="n">
-        <v>0.176</v>
+        <v>0.961</v>
       </c>
     </row>
     <row r="21">
@@ -3130,13 +3132,13 @@
         <v>2031</v>
       </c>
       <c r="B21" t="n">
-        <v>0.483</v>
+        <v>2.222</v>
       </c>
       <c r="C21" t="n">
         <v>0.5204</v>
       </c>
       <c r="D21" t="n">
-        <v>0.251</v>
+        <v>1.156</v>
       </c>
     </row>
     <row r="22">
@@ -3144,13 +3146,13 @@
         <v>2032</v>
       </c>
       <c r="B22" t="n">
-        <v>0.717</v>
+        <v>2.758</v>
       </c>
       <c r="C22" t="n">
         <v>0.4667</v>
       </c>
       <c r="D22" t="n">
-        <v>0.335</v>
+        <v>1.287</v>
       </c>
     </row>
     <row r="23">
@@ -3158,13 +3160,13 @@
         <v>2033</v>
       </c>
       <c r="B23" t="n">
-        <v>0.883</v>
+        <v>3.284</v>
       </c>
       <c r="C23" t="n">
         <v>0.4186</v>
       </c>
       <c r="D23" t="n">
-        <v>0.37</v>
+        <v>1.375</v>
       </c>
     </row>
     <row r="24">
@@ -3172,13 +3174,13 @@
         <v>2034</v>
       </c>
       <c r="B24" t="n">
-        <v>1.097</v>
+        <v>3.698</v>
       </c>
       <c r="C24" t="n">
         <v>0.3754</v>
       </c>
       <c r="D24" t="n">
-        <v>0.412</v>
+        <v>1.388</v>
       </c>
     </row>
     <row r="25">
@@ -3186,13 +3188,13 @@
         <v>2035</v>
       </c>
       <c r="B25" t="n">
-        <v>1.239</v>
+        <v>4.11</v>
       </c>
       <c r="C25" t="n">
         <v>0.3367</v>
       </c>
       <c r="D25" t="n">
-        <v>0.417</v>
+        <v>1.384</v>
       </c>
     </row>
     <row r="26">
@@ -3203,7 +3205,7 @@
       </c>
       <c r="D26" s="22" t="inlineStr">
         <is>
-          <t>1.780B</t>
+          <t>7.855B</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3254,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>1.239B</t>
+          <t>4.110B</t>
         </is>
       </c>
     </row>
@@ -3264,12 +3266,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>1.239 x (1 + 0.0350)</t>
+          <t>4.110 x (1 + 0.0350)</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>1.282B</t>
+          <t>4.253B</t>
         </is>
       </c>
     </row>
@@ -3281,12 +3283,12 @@
       </c>
       <c r="B33" s="21" t="inlineStr">
         <is>
-          <t>1.282 / (0.1150 - 0.0350)</t>
+          <t>4.253 / (0.1150 - 0.0350)</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>16.031B</t>
+          <t>53.168B</t>
         </is>
       </c>
     </row>
@@ -3298,12 +3300,12 @@
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>16.031 / (1+0.1150)^10</t>
+          <t>53.168 / (1+0.1150)^10</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>5.398B</t>
+          <t>17.902B</t>
         </is>
       </c>
     </row>
@@ -3347,12 +3349,12 @@
       </c>
       <c r="B39" s="21" t="inlineStr">
         <is>
-          <t>1.780 + 5.398</t>
+          <t>7.855 + 17.902</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>7.178B</t>
+          <t>25.757B</t>
         </is>
       </c>
     </row>
@@ -3364,12 +3366,12 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>7.178 - -0.439</t>
+          <t>25.757 - -0.439</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>7.617B</t>
+          <t>26.196B</t>
         </is>
       </c>
     </row>
@@ -3381,12 +3383,12 @@
       </c>
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>7.617B / 0.220B shares</t>
+          <t>26.196B / 0.220B shares</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>$34.69</t>
+          <t>$119.29</t>
         </is>
       </c>
     </row>
@@ -3469,19 +3471,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37.4</v>
+        <v>128.69</v>
       </c>
       <c r="C4" t="n">
-        <v>39.32</v>
+        <v>135.03</v>
       </c>
       <c r="D4" t="n">
-        <v>41.5</v>
+        <v>142.29</v>
       </c>
       <c r="E4" t="n">
-        <v>44.03</v>
+        <v>150.66</v>
       </c>
       <c r="F4" t="n">
-        <v>46.97</v>
+        <v>160.43</v>
       </c>
     </row>
     <row r="5">
@@ -3491,19 +3493,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>34.39</v>
+        <v>118.51</v>
       </c>
       <c r="C5" t="n">
-        <v>36.01</v>
+        <v>123.88</v>
       </c>
       <c r="D5" t="n">
-        <v>37.85</v>
+        <v>129.98</v>
       </c>
       <c r="E5" t="n">
-        <v>39.95</v>
+        <v>136.95</v>
       </c>
       <c r="F5" t="n">
-        <v>42.38</v>
+        <v>144.99</v>
       </c>
     </row>
     <row r="6">
@@ -3513,19 +3515,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>31.74</v>
+        <v>109.53</v>
       </c>
       <c r="C6" t="n">
-        <v>33.13</v>
+        <v>114.12</v>
       </c>
       <c r="D6" t="n">
-        <v>34.69</v>
+        <v>119.29</v>
       </c>
       <c r="E6" t="n">
-        <v>36.45</v>
+        <v>125.14</v>
       </c>
       <c r="F6" t="n">
-        <v>38.47</v>
+        <v>131.83</v>
       </c>
     </row>
     <row r="7">
@@ -3535,19 +3537,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29.4</v>
+        <v>101.57</v>
       </c>
       <c r="C7" t="n">
-        <v>30.59</v>
+        <v>105.51</v>
       </c>
       <c r="D7" t="n">
-        <v>31.92</v>
+        <v>109.92</v>
       </c>
       <c r="E7" t="n">
-        <v>33.41</v>
+        <v>114.89</v>
       </c>
       <c r="F7" t="n">
-        <v>35.11</v>
+        <v>120.51</v>
       </c>
     </row>
     <row r="8">
@@ -3557,19 +3559,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>27.31</v>
+        <v>94.45999999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>28.34</v>
+        <v>97.87</v>
       </c>
       <c r="D8" t="n">
-        <v>29.48</v>
+        <v>101.66</v>
       </c>
       <c r="E8" t="n">
-        <v>30.76</v>
+        <v>105.9</v>
       </c>
       <c r="F8" t="n">
-        <v>32.2</v>
+        <v>110.67</v>
       </c>
     </row>
   </sheetData>
@@ -3812,14 +3814,14 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>109.36</v>
+        <v>193.26</v>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>EV/Sales is the standard cross-check for loss-making hypergrowth. Peer set: high-growth AI compute and inference names. A rich 28x FY26E sales is generous versus where most AI hardware trades, and still implies a price far below the current $237.83, underscoring how stretched the trailing 102x multiple is.</t>
+          <t>UBS values CBRS at 10x EV/Sales on C2029E sales discounted back. We apply the same compute-peer ~10x multiple but to our risk-adjusted C2028E sales of $4.2B, undiscounted, as a ~18-month forward target proxy. This stays conservative versus UBS (lower year, lower sales) while using the same relative lens the market is using.</t>
         </is>
       </c>
     </row>
@@ -3904,22 +3906,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15.41</v>
+        <v>39.53</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="D5" t="n">
-        <v>3.08</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Meaningful odds. The G42 concentration, export-control exposure and the IPO lock-up unlock against a 8.67M-share float are concrete, dateable downside catalysts, not tail risks.</t>
+          <t>Real odds. The OpenAI ramp depends on scaling supply ~10x; NVDA folding Groq into its roadmap could take the ultra-fast-inference niche; the deal is concentrated and the lock-up unlock still looms. Any one slips the model badly.</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Growth decelerates hard as Condor Galaxy installs lap, a token price war caps margins, and the unlock floods supply.</t>
+          <t>OpenAI deployment stalls or NVDA/Groq wins the segment; revenue lands far below the risk-adjusted base and the multiple compresses.</t>
         </is>
       </c>
     </row>
@@ -3930,22 +3932,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>34.69</v>
+        <v>119.29</v>
       </c>
       <c r="C6" s="11" t="n">
         <v>0.45</v>
       </c>
       <c r="D6" t="n">
-        <v>15.61</v>
+        <v>53.68</v>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Central case. Revenue keeps compounding fast and the company reaches operating profit around 2028, but the stock is valued far ahead of even this constructive ramp.</t>
+          <t>Central case. OpenAI deploys but a year behind UBS at ~55-60% utilization; AWS stays optional. Most likely path given execution risk on a 10x scale-up.</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Strong execution on inference and diversification, with FCF margin reaching the mid-20s by the early 2030s.</t>
+          <t>Risk-adjusted OpenAI ramp to ~$8.5B revenue by 2030 at hardware-like margins.</t>
         </is>
       </c>
     </row>
@@ -3956,22 +3958,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>67.20999999999999</v>
+        <v>255.49</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="D7" t="n">
-        <v>10.08</v>
+        <v>51.1</v>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Lower odds. Requires inference demand to reaccelerate revenue, margins to expand faster than modeled, and concentration to resolve cleanly before the unlock.</t>
+          <t>Plausible. If OpenAI ramps on UBS's schedule and AWS scales into a multi-billion hardware stream, revenue approaches UBS's $11B+ 2029 and margins hit the high-30s.</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Cerebras becomes the default fast-inference layer; revenue and FCF margins beat the base path materially.</t>
+          <t>OpenAI on schedule plus AWS optionality converting; trajectory approaches the UBS base.</t>
         </is>
       </c>
     </row>
@@ -3982,17 +3984,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>109.36</v>
+        <v>193.26</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D8" t="n">
-        <v>21.87</v>
+        <v>19.33</v>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>EV/Sales is the standard cross-check for loss-making hypergrowth. Peer set: high-growth AI compute and inference names. A rich 28x FY26E sales is generous versus where most AI hardware trades, and still implies a price far below the current $237.83, underscoring how stretched the trailing 102x multiple is.</t>
+          <t>UBS values CBRS at 10x EV/Sales on C2029E sales discounted back. We apply the same compute-peer ~10x multiple but to our risk-adjusted C2028E sales of $4.2B, undiscounted, as a ~18-month forward target proxy. This stays conservative versus UBS (lower year, lower sales) while using the same relative lens the market is using.</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -4019,7 +4021,7 @@
         </is>
       </c>
       <c r="D11" s="19" t="n">
-        <v>50.64</v>
+        <v>133.99</v>
       </c>
     </row>
     <row r="12">
@@ -4039,7 +4041,7 @@
         </is>
       </c>
       <c r="D13" s="25" t="n">
-        <v>-0.787</v>
+        <v>-0.4370000000000001</v>
       </c>
     </row>
     <row r="14"/>
@@ -4054,7 +4056,7 @@
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Base 45% reflects a constructive but realistic ramp. Bear gets a heavy 20% because the lock-up unlock, G42 concentration and export risk are concrete near-term catalysts, not tail events. Bull 15% for the demand-reacceleration case. The EV/Sales cross-check carries 20% to anchor against intrinsic value with a relative lens; notably even a generous 28x sales multiple lands well below spot, which is the central finding.</t>
+          <t>Base 45% on the risk-adjusted OpenAI ramp. Bear gets a heavy 25% because the 10x supply-chain scale-up, OpenAI concentration, NVDA/Groq competitive response, and the IPO lock-up are all live. Bull 20% for the OpenAI-on-schedule-plus-AWS case. Cross-check 10% as a hardware-peer relative anchor. The blend deliberately stays below UBS's $300 by haircutting the deal for execution rather than disputing the technology.</t>
         </is>
       </c>
     </row>

</xml_diff>